<commit_message>
style(despesas): refine checkbox UI, selection feedback and thumbnail borders
</commit_message>
<xml_diff>
--- a/RDT.xlsx
+++ b/RDT.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lucas\OneDrive\Desktop\Lucas\BBTS\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lucas\OneDrive\Desktop\Lucas\Projetos\RDT App\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9F95E5B1-3F7C-42E3-82F9-6E339CD482CA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1EEDA16B-1098-4150-BA8A-B882F5D26B84}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -139,7 +139,7 @@
     <numFmt numFmtId="164" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* \-??_);_(@_)"/>
     <numFmt numFmtId="165" formatCode="000"/>
   </numFmts>
-  <fonts count="20" x14ac:knownFonts="1">
+  <fonts count="21" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -262,6 +262,12 @@
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="5">
@@ -473,7 +479,7 @@
     <xf numFmtId="164" fontId="17" fillId="0" borderId="0" applyBorder="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="89">
+  <cellXfs count="90">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -653,6 +659,7 @@
     <xf numFmtId="0" fontId="11" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="2" applyFont="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1332,7 +1339,7 @@
     </row>
     <row r="13" spans="1:9" s="30" customFormat="1" ht="23.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="83"/>
-      <c r="B13" s="83"/>
+      <c r="B13" s="89"/>
       <c r="C13" s="38"/>
       <c r="D13" s="83"/>
       <c r="E13" s="40"/>

</xml_diff>

<commit_message>
chore: update build artifacts and data files
</commit_message>
<xml_diff>
--- a/RDT.xlsx
+++ b/RDT.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lucas\OneDrive\Desktop\Lucas\Projetos\RDT App\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1EEDA16B-1098-4150-BA8A-B882F5D26B84}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{92976F93-3986-4B30-937E-DDDBAEA6FE2A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -479,7 +479,7 @@
     <xf numFmtId="164" fontId="17" fillId="0" borderId="0" applyBorder="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="90">
+  <cellXfs count="91">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -513,7 +513,6 @@
     <xf numFmtId="0" fontId="7" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -645,7 +644,7 @@
     <xf numFmtId="0" fontId="15" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="18" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="2"/>
-    <xf numFmtId="49" fontId="19" fillId="0" borderId="0" xfId="2" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="2" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
       <protection locked="0"/>
@@ -659,7 +658,9 @@
     <xf numFmtId="0" fontId="11" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="2" applyFont="1"/>
+    <xf numFmtId="49" fontId="19" fillId="0" borderId="10" xfId="2" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="10" xfId="2" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1182,13 +1183,13 @@
   <sheetData>
     <row r="1" spans="1:9" s="4" customFormat="1" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C1" s="5"/>
-      <c r="D1" s="85" t="s">
-        <v>0</v>
-      </c>
-      <c r="E1" s="85"/>
-      <c r="F1" s="85"/>
-      <c r="G1" s="85"/>
-      <c r="H1" s="85"/>
+      <c r="D1" s="84" t="s">
+        <v>0</v>
+      </c>
+      <c r="E1" s="84"/>
+      <c r="F1" s="84"/>
+      <c r="G1" s="84"/>
+      <c r="H1" s="84"/>
     </row>
     <row r="2" spans="1:9" s="4" customFormat="1" ht="15" x14ac:dyDescent="0.2">
       <c r="C2" s="6"/>
@@ -1238,22 +1239,23 @@
       <c r="I5" s="23"/>
     </row>
     <row r="6" spans="1:9" s="16" customFormat="1" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="24" t="s">
+      <c r="A6" s="15" t="s">
         <v>4</v>
       </c>
-      <c r="D6" s="25"/>
+      <c r="D6" s="24"/>
       <c r="E6" s="16" t="s">
         <v>5</v>
       </c>
-      <c r="F6" s="26"/>
-      <c r="I6" s="27"/>
+      <c r="F6" s="25"/>
+      <c r="I6" s="26"/>
     </row>
     <row r="7" spans="1:9" s="16" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B7" s="18"/>
-      <c r="C7" s="82" t="s">
+      <c r="A7" s="90"/>
+      <c r="B7" s="19"/>
+      <c r="C7" s="81" t="s">
         <v>27</v>
       </c>
-      <c r="D7" s="28"/>
+      <c r="D7" s="27"/>
       <c r="E7" s="19">
         <v>7281</v>
       </c>
@@ -1265,34 +1267,34 @@
     <row r="8" spans="1:9" s="16" customFormat="1" ht="8.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="D8" s="17"/>
     </row>
-    <row r="9" spans="1:9" s="30" customFormat="1" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:9" s="29" customFormat="1" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="B9" s="86" t="s">
+      <c r="B9" s="85" t="s">
         <v>7</v>
       </c>
-      <c r="C9" s="86"/>
-      <c r="D9" s="29" t="s">
+      <c r="C9" s="85"/>
+      <c r="D9" s="28" t="s">
         <v>30</v>
       </c>
-      <c r="E9" s="87" t="s">
+      <c r="E9" s="86" t="s">
         <v>8</v>
       </c>
-      <c r="F9" s="87"/>
-      <c r="G9" s="87"/>
-      <c r="H9" s="29" t="s">
+      <c r="F9" s="86"/>
+      <c r="G9" s="86"/>
+      <c r="H9" s="28" t="s">
         <v>9</v>
       </c>
-      <c r="I9" s="29" t="s">
+      <c r="I9" s="28" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="10" spans="1:9" s="30" customFormat="1" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="31"/>
-      <c r="B10" s="32"/>
-      <c r="C10" s="33"/>
-      <c r="D10" s="34"/>
+    <row r="10" spans="1:9" s="29" customFormat="1" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A10" s="30"/>
+      <c r="B10" s="31"/>
+      <c r="C10" s="32"/>
+      <c r="D10" s="33"/>
       <c r="E10" s="1" t="s">
         <v>11</v>
       </c>
@@ -1302,341 +1304,341 @@
       <c r="G10" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="H10" s="35"/>
-      <c r="I10" s="35"/>
-    </row>
-    <row r="11" spans="1:9" s="30" customFormat="1" ht="23.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="84"/>
-      <c r="B11" s="37"/>
-      <c r="C11" s="38"/>
-      <c r="D11" s="44"/>
-      <c r="E11" s="40"/>
-      <c r="F11" s="40"/>
-      <c r="G11" s="41">
+      <c r="H10" s="34"/>
+      <c r="I10" s="34"/>
+    </row>
+    <row r="11" spans="1:9" s="29" customFormat="1" ht="23.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="88"/>
+      <c r="B11" s="36"/>
+      <c r="C11" s="37"/>
+      <c r="D11" s="43"/>
+      <c r="E11" s="39"/>
+      <c r="F11" s="39"/>
+      <c r="G11" s="40">
         <f>E11*F11</f>
         <v>0</v>
       </c>
-      <c r="H11" s="41">
-        <v>0</v>
-      </c>
-      <c r="I11" s="42">
+      <c r="H11" s="40">
+        <v>0</v>
+      </c>
+      <c r="I11" s="41">
         <f>G11+H11</f>
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:9" s="30" customFormat="1" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="43" t="s">
+    <row r="12" spans="1:9" s="29" customFormat="1" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A12" s="42" t="s">
         <v>14</v>
       </c>
-      <c r="B12" s="44"/>
-      <c r="C12" s="44"/>
-      <c r="D12" s="45"/>
-      <c r="E12" s="44"/>
-      <c r="F12" s="44"/>
-      <c r="G12" s="44"/>
-      <c r="H12" s="46"/>
-      <c r="I12" s="47"/>
-    </row>
-    <row r="13" spans="1:9" s="30" customFormat="1" ht="23.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="83"/>
-      <c r="B13" s="89"/>
-      <c r="C13" s="38"/>
-      <c r="D13" s="83"/>
-      <c r="E13" s="40"/>
-      <c r="F13" s="40"/>
-      <c r="G13" s="41">
+      <c r="B12" s="43"/>
+      <c r="C12" s="43"/>
+      <c r="D12" s="44"/>
+      <c r="E12" s="43"/>
+      <c r="F12" s="43"/>
+      <c r="G12" s="43"/>
+      <c r="H12" s="45"/>
+      <c r="I12" s="46"/>
+    </row>
+    <row r="13" spans="1:9" s="29" customFormat="1" ht="23.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="89"/>
+      <c r="B13" s="83"/>
+      <c r="C13" s="37"/>
+      <c r="D13" s="82"/>
+      <c r="E13" s="39"/>
+      <c r="F13" s="39"/>
+      <c r="G13" s="40">
         <f>E13*F13</f>
         <v>0</v>
       </c>
-      <c r="H13" s="41">
-        <v>0</v>
-      </c>
-      <c r="I13" s="42">
+      <c r="H13" s="40">
+        <v>0</v>
+      </c>
+      <c r="I13" s="41">
         <f>G13+H13</f>
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:9" s="30" customFormat="1" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="43" t="s">
+    <row r="14" spans="1:9" s="29" customFormat="1" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A14" s="42" t="s">
         <v>14</v>
       </c>
-      <c r="B14" s="44"/>
-      <c r="C14" s="44"/>
-      <c r="D14" s="45"/>
-      <c r="E14" s="44"/>
-      <c r="F14" s="44"/>
-      <c r="G14" s="44"/>
-      <c r="H14" s="46"/>
-      <c r="I14" s="47"/>
-    </row>
-    <row r="15" spans="1:9" s="30" customFormat="1" ht="23.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="83"/>
-      <c r="B15" s="37"/>
-      <c r="C15" s="38"/>
-      <c r="D15" s="39"/>
-      <c r="E15" s="40"/>
-      <c r="F15" s="40"/>
-      <c r="G15" s="41">
+      <c r="B14" s="43"/>
+      <c r="C14" s="43"/>
+      <c r="D14" s="44"/>
+      <c r="E14" s="43"/>
+      <c r="F14" s="43"/>
+      <c r="G14" s="43"/>
+      <c r="H14" s="45"/>
+      <c r="I14" s="46"/>
+    </row>
+    <row r="15" spans="1:9" s="29" customFormat="1" ht="23.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="89"/>
+      <c r="B15" s="36"/>
+      <c r="C15" s="37"/>
+      <c r="D15" s="38"/>
+      <c r="E15" s="39"/>
+      <c r="F15" s="39"/>
+      <c r="G15" s="40">
         <f>E15*F15</f>
         <v>0</v>
       </c>
-      <c r="H15" s="41">
-        <v>0</v>
-      </c>
-      <c r="I15" s="42">
+      <c r="H15" s="40">
+        <v>0</v>
+      </c>
+      <c r="I15" s="41">
         <f>G15+H15</f>
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:9" s="30" customFormat="1" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="43" t="s">
+    <row r="16" spans="1:9" s="29" customFormat="1" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A16" s="42" t="s">
         <v>14</v>
       </c>
-      <c r="B16" s="44"/>
-      <c r="C16" s="44"/>
-      <c r="D16" s="45"/>
-      <c r="E16" s="44"/>
-      <c r="F16" s="44"/>
-      <c r="G16" s="44"/>
-      <c r="H16" s="46"/>
-      <c r="I16" s="47"/>
-    </row>
-    <row r="17" spans="1:9" s="30" customFormat="1" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="36"/>
-      <c r="B17" s="37"/>
-      <c r="C17" s="38"/>
-      <c r="D17" s="39"/>
-      <c r="E17" s="40"/>
-      <c r="F17" s="40"/>
-      <c r="G17" s="41">
+      <c r="B16" s="43"/>
+      <c r="C16" s="43"/>
+      <c r="D16" s="44"/>
+      <c r="E16" s="43"/>
+      <c r="F16" s="43"/>
+      <c r="G16" s="43"/>
+      <c r="H16" s="45"/>
+      <c r="I16" s="46"/>
+    </row>
+    <row r="17" spans="1:9" s="29" customFormat="1" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A17" s="35"/>
+      <c r="B17" s="36"/>
+      <c r="C17" s="37"/>
+      <c r="D17" s="38"/>
+      <c r="E17" s="39"/>
+      <c r="F17" s="39"/>
+      <c r="G17" s="40">
         <f>E17*F17</f>
         <v>0</v>
       </c>
-      <c r="H17" s="41">
-        <v>0</v>
-      </c>
-      <c r="I17" s="42">
+      <c r="H17" s="40">
+        <v>0</v>
+      </c>
+      <c r="I17" s="41">
         <f>G17+H17</f>
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:9" s="30" customFormat="1" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="43" t="s">
+    <row r="18" spans="1:9" s="29" customFormat="1" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A18" s="42" t="s">
         <v>14</v>
       </c>
-      <c r="B18" s="44"/>
-      <c r="C18" s="44"/>
-      <c r="D18" s="45"/>
-      <c r="E18" s="44"/>
-      <c r="F18" s="44"/>
-      <c r="G18" s="44"/>
-      <c r="H18" s="46"/>
-      <c r="I18" s="47"/>
-    </row>
-    <row r="19" spans="1:9" s="30" customFormat="1" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A19" s="36"/>
-      <c r="B19" s="37"/>
-      <c r="C19" s="38"/>
-      <c r="D19" s="39"/>
-      <c r="E19" s="40"/>
-      <c r="F19" s="40"/>
-      <c r="G19" s="41">
+      <c r="B18" s="43"/>
+      <c r="C18" s="43"/>
+      <c r="D18" s="44"/>
+      <c r="E18" s="43"/>
+      <c r="F18" s="43"/>
+      <c r="G18" s="43"/>
+      <c r="H18" s="45"/>
+      <c r="I18" s="46"/>
+    </row>
+    <row r="19" spans="1:9" s="29" customFormat="1" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A19" s="35"/>
+      <c r="B19" s="36"/>
+      <c r="C19" s="37"/>
+      <c r="D19" s="38"/>
+      <c r="E19" s="39"/>
+      <c r="F19" s="39"/>
+      <c r="G19" s="40">
         <f>E19*F19</f>
         <v>0</v>
       </c>
-      <c r="H19" s="41">
-        <v>0</v>
-      </c>
-      <c r="I19" s="42">
+      <c r="H19" s="40">
+        <v>0</v>
+      </c>
+      <c r="I19" s="41">
         <f>G19+H19</f>
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:9" s="30" customFormat="1" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A20" s="43" t="s">
+    <row r="20" spans="1:9" s="29" customFormat="1" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A20" s="42" t="s">
         <v>14</v>
       </c>
-      <c r="B20" s="44"/>
-      <c r="C20" s="44"/>
-      <c r="D20" s="45"/>
-      <c r="E20" s="44"/>
-      <c r="F20" s="44"/>
-      <c r="G20" s="44"/>
-      <c r="H20" s="46"/>
-      <c r="I20" s="47"/>
-    </row>
-    <row r="21" spans="1:9" s="30" customFormat="1" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A21" s="36"/>
-      <c r="B21" s="37"/>
-      <c r="C21" s="38"/>
-      <c r="D21" s="39"/>
-      <c r="E21" s="40"/>
-      <c r="F21" s="40"/>
-      <c r="G21" s="41">
+      <c r="B20" s="43"/>
+      <c r="C20" s="43"/>
+      <c r="D20" s="44"/>
+      <c r="E20" s="43"/>
+      <c r="F20" s="43"/>
+      <c r="G20" s="43"/>
+      <c r="H20" s="45"/>
+      <c r="I20" s="46"/>
+    </row>
+    <row r="21" spans="1:9" s="29" customFormat="1" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A21" s="35"/>
+      <c r="B21" s="36"/>
+      <c r="C21" s="37"/>
+      <c r="D21" s="38"/>
+      <c r="E21" s="39"/>
+      <c r="F21" s="39"/>
+      <c r="G21" s="40">
         <f>E21*F21</f>
         <v>0</v>
       </c>
-      <c r="H21" s="41">
-        <v>0</v>
-      </c>
-      <c r="I21" s="42">
+      <c r="H21" s="40">
+        <v>0</v>
+      </c>
+      <c r="I21" s="41">
         <f>G21+H21</f>
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:9" s="30" customFormat="1" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="43" t="s">
+    <row r="22" spans="1:9" s="29" customFormat="1" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A22" s="42" t="s">
         <v>14</v>
       </c>
-      <c r="B22" s="44"/>
-      <c r="C22" s="44"/>
-      <c r="D22" s="45"/>
-      <c r="E22" s="44"/>
-      <c r="F22" s="44"/>
-      <c r="G22" s="44"/>
-      <c r="H22" s="46"/>
-      <c r="I22" s="47"/>
-    </row>
-    <row r="23" spans="1:9" s="30" customFormat="1" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A23" s="36"/>
-      <c r="B23" s="37"/>
-      <c r="C23" s="38"/>
-      <c r="D23" s="39"/>
-      <c r="E23" s="40"/>
-      <c r="F23" s="40"/>
-      <c r="G23" s="41">
+      <c r="B22" s="43"/>
+      <c r="C22" s="43"/>
+      <c r="D22" s="44"/>
+      <c r="E22" s="43"/>
+      <c r="F22" s="43"/>
+      <c r="G22" s="43"/>
+      <c r="H22" s="45"/>
+      <c r="I22" s="46"/>
+    </row>
+    <row r="23" spans="1:9" s="29" customFormat="1" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A23" s="35"/>
+      <c r="B23" s="36"/>
+      <c r="C23" s="37"/>
+      <c r="D23" s="38"/>
+      <c r="E23" s="39"/>
+      <c r="F23" s="39"/>
+      <c r="G23" s="40">
         <f>E23*F23</f>
         <v>0</v>
       </c>
-      <c r="H23" s="41">
-        <v>0</v>
-      </c>
-      <c r="I23" s="42">
+      <c r="H23" s="40">
+        <v>0</v>
+      </c>
+      <c r="I23" s="41">
         <f>G23+H23</f>
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:9" s="30" customFormat="1" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A24" s="43" t="s">
+    <row r="24" spans="1:9" s="29" customFormat="1" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A24" s="42" t="s">
         <v>14</v>
       </c>
-      <c r="B24" s="44"/>
-      <c r="C24" s="44"/>
-      <c r="D24" s="45"/>
-      <c r="E24" s="44"/>
-      <c r="F24" s="44"/>
-      <c r="G24" s="44"/>
-      <c r="H24" s="46"/>
-      <c r="I24" s="47"/>
-    </row>
-    <row r="25" spans="1:9" s="30" customFormat="1" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A25" s="36"/>
-      <c r="B25" s="37"/>
-      <c r="C25" s="38"/>
-      <c r="D25" s="39"/>
-      <c r="E25" s="40"/>
-      <c r="F25" s="40"/>
-      <c r="G25" s="41">
+      <c r="B24" s="43"/>
+      <c r="C24" s="43"/>
+      <c r="D24" s="44"/>
+      <c r="E24" s="43"/>
+      <c r="F24" s="43"/>
+      <c r="G24" s="43"/>
+      <c r="H24" s="45"/>
+      <c r="I24" s="46"/>
+    </row>
+    <row r="25" spans="1:9" s="29" customFormat="1" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A25" s="35"/>
+      <c r="B25" s="36"/>
+      <c r="C25" s="37"/>
+      <c r="D25" s="38"/>
+      <c r="E25" s="39"/>
+      <c r="F25" s="39"/>
+      <c r="G25" s="40">
         <f>E25*F25</f>
         <v>0</v>
       </c>
-      <c r="H25" s="41">
-        <v>0</v>
-      </c>
-      <c r="I25" s="42">
+      <c r="H25" s="40">
+        <v>0</v>
+      </c>
+      <c r="I25" s="41">
         <f>G25+H25</f>
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:9" s="30" customFormat="1" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A26" s="43" t="s">
+    <row r="26" spans="1:9" s="29" customFormat="1" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A26" s="42" t="s">
         <v>14</v>
       </c>
-      <c r="B26" s="44"/>
-      <c r="C26" s="44"/>
-      <c r="D26" s="45"/>
-      <c r="E26" s="44"/>
-      <c r="F26" s="44"/>
-      <c r="G26" s="44"/>
-      <c r="H26" s="46"/>
-      <c r="I26" s="47"/>
-    </row>
-    <row r="27" spans="1:9" s="30" customFormat="1" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A27" s="36"/>
-      <c r="B27" s="37"/>
-      <c r="C27" s="38"/>
-      <c r="D27" s="39"/>
-      <c r="E27" s="40"/>
-      <c r="F27" s="40"/>
-      <c r="G27" s="41">
+      <c r="B26" s="43"/>
+      <c r="C26" s="43"/>
+      <c r="D26" s="44"/>
+      <c r="E26" s="43"/>
+      <c r="F26" s="43"/>
+      <c r="G26" s="43"/>
+      <c r="H26" s="45"/>
+      <c r="I26" s="46"/>
+    </row>
+    <row r="27" spans="1:9" s="29" customFormat="1" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A27" s="35"/>
+      <c r="B27" s="36"/>
+      <c r="C27" s="37"/>
+      <c r="D27" s="38"/>
+      <c r="E27" s="39"/>
+      <c r="F27" s="39"/>
+      <c r="G27" s="40">
         <f>E27*F27</f>
         <v>0</v>
       </c>
-      <c r="H27" s="41">
-        <v>0</v>
-      </c>
-      <c r="I27" s="42">
+      <c r="H27" s="40">
+        <v>0</v>
+      </c>
+      <c r="I27" s="41">
         <f>G27+H27</f>
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:9" s="30" customFormat="1" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A28" s="43" t="s">
+    <row r="28" spans="1:9" s="29" customFormat="1" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A28" s="42" t="s">
         <v>14</v>
       </c>
-      <c r="B28" s="44"/>
-      <c r="C28" s="44"/>
-      <c r="D28" s="45"/>
-      <c r="E28" s="44"/>
-      <c r="F28" s="44"/>
-      <c r="G28" s="44"/>
-      <c r="H28" s="46"/>
-      <c r="I28" s="47"/>
-    </row>
-    <row r="29" spans="1:9" s="30" customFormat="1" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A29" s="36"/>
-      <c r="B29" s="37"/>
-      <c r="C29" s="38"/>
-      <c r="D29" s="39"/>
-      <c r="E29" s="40"/>
-      <c r="F29" s="40"/>
-      <c r="G29" s="41">
+      <c r="B28" s="43"/>
+      <c r="C28" s="43"/>
+      <c r="D28" s="44"/>
+      <c r="E28" s="43"/>
+      <c r="F28" s="43"/>
+      <c r="G28" s="43"/>
+      <c r="H28" s="45"/>
+      <c r="I28" s="46"/>
+    </row>
+    <row r="29" spans="1:9" s="29" customFormat="1" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A29" s="35"/>
+      <c r="B29" s="36"/>
+      <c r="C29" s="37"/>
+      <c r="D29" s="38"/>
+      <c r="E29" s="39"/>
+      <c r="F29" s="39"/>
+      <c r="G29" s="40">
         <f>E29*F29</f>
         <v>0</v>
       </c>
-      <c r="H29" s="41">
-        <v>0</v>
-      </c>
-      <c r="I29" s="42">
+      <c r="H29" s="40">
+        <v>0</v>
+      </c>
+      <c r="I29" s="41">
         <f>G29+H29</f>
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="1:9" s="30" customFormat="1" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A30" s="43" t="s">
+    <row r="30" spans="1:9" s="29" customFormat="1" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A30" s="42" t="s">
         <v>14</v>
       </c>
-      <c r="B30" s="44"/>
-      <c r="C30" s="44"/>
-      <c r="D30" s="45"/>
-      <c r="E30" s="44"/>
-      <c r="F30" s="44"/>
-      <c r="G30" s="44"/>
-      <c r="H30" s="46"/>
-      <c r="I30" s="47"/>
-    </row>
-    <row r="31" spans="1:9" s="30" customFormat="1" ht="23.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="88" t="s">
+      <c r="B30" s="43"/>
+      <c r="C30" s="43"/>
+      <c r="D30" s="44"/>
+      <c r="E30" s="43"/>
+      <c r="F30" s="43"/>
+      <c r="G30" s="43"/>
+      <c r="H30" s="45"/>
+      <c r="I30" s="46"/>
+    </row>
+    <row r="31" spans="1:9" s="29" customFormat="1" ht="23.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A31" s="87" t="s">
         <v>15</v>
       </c>
-      <c r="B31" s="88"/>
-      <c r="C31" s="88"/>
-      <c r="D31" s="88"/>
-      <c r="E31" s="88"/>
-      <c r="F31" s="88"/>
-      <c r="G31" s="88"/>
-      <c r="H31" s="88"/>
-      <c r="I31" s="48">
+      <c r="B31" s="87"/>
+      <c r="C31" s="87"/>
+      <c r="D31" s="87"/>
+      <c r="E31" s="87"/>
+      <c r="F31" s="87"/>
+      <c r="G31" s="87"/>
+      <c r="H31" s="87"/>
+      <c r="I31" s="47">
         <f>SUM(I11,I13,I15,I17,I19,I21,I23,I25,I27,I29)</f>
         <v>0</v>
       </c>
@@ -1644,100 +1646,100 @@
     <row r="32" spans="1:9" s="16" customFormat="1" ht="12" customHeight="1" x14ac:dyDescent="0.2">
       <c r="D32" s="17"/>
     </row>
-    <row r="33" spans="1:10" s="50" customFormat="1" ht="10.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A33" s="49"/>
-      <c r="B33" s="49"/>
-      <c r="D33" s="51"/>
-      <c r="E33" s="52" t="s">
+    <row r="33" spans="1:10" s="49" customFormat="1" ht="10.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A33" s="48"/>
+      <c r="B33" s="48"/>
+      <c r="D33" s="50"/>
+      <c r="E33" s="51" t="s">
         <v>16</v>
       </c>
-      <c r="F33" s="53"/>
-      <c r="G33" s="54"/>
-      <c r="H33" s="55"/>
-      <c r="I33" s="56"/>
-      <c r="J33" s="57"/>
-    </row>
-    <row r="34" spans="1:10" s="50" customFormat="1" ht="10.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A34" s="49" t="s">
+      <c r="F33" s="52"/>
+      <c r="G33" s="53"/>
+      <c r="H33" s="54"/>
+      <c r="I33" s="55"/>
+      <c r="J33" s="56"/>
+    </row>
+    <row r="34" spans="1:10" s="49" customFormat="1" ht="10.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A34" s="48" t="s">
         <v>17</v>
       </c>
-      <c r="B34" s="58" t="s">
+      <c r="B34" s="57" t="s">
         <v>18</v>
       </c>
-      <c r="C34" s="59" t="s">
+      <c r="C34" s="58" t="s">
         <v>19</v>
       </c>
-      <c r="D34" s="60"/>
-      <c r="E34" s="55" t="s">
+      <c r="D34" s="59"/>
+      <c r="E34" s="54" t="s">
         <v>20</v>
       </c>
-      <c r="F34" s="61"/>
-      <c r="G34" s="56"/>
-      <c r="H34" s="55" t="s">
+      <c r="F34" s="60"/>
+      <c r="G34" s="55"/>
+      <c r="H34" s="54" t="s">
         <v>21</v>
       </c>
-      <c r="I34" s="56"/>
-      <c r="J34" s="57"/>
-    </row>
-    <row r="35" spans="1:10" s="50" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A35" s="62">
+      <c r="I34" s="55"/>
+      <c r="J34" s="56"/>
+    </row>
+    <row r="35" spans="1:10" s="49" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A35" s="61">
         <v>1</v>
       </c>
-      <c r="B35" s="63" t="s">
+      <c r="B35" s="62" t="s">
         <v>28</v>
       </c>
-      <c r="C35" s="64" t="s">
+      <c r="C35" s="63" t="s">
         <v>29</v>
       </c>
-      <c r="D35" s="65"/>
-      <c r="E35" s="66"/>
-      <c r="F35" s="67"/>
-      <c r="G35" s="67"/>
-      <c r="H35" s="68"/>
-      <c r="I35" s="69"/>
-      <c r="J35" s="57"/>
+      <c r="D35" s="64"/>
+      <c r="E35" s="65"/>
+      <c r="F35" s="66"/>
+      <c r="G35" s="66"/>
+      <c r="H35" s="67"/>
+      <c r="I35" s="68"/>
+      <c r="J35" s="56"/>
     </row>
     <row r="36" spans="1:10" s="16" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A36" s="70" t="s">
+      <c r="A36" s="69" t="s">
         <v>22</v>
       </c>
       <c r="D36" s="17"/>
-      <c r="E36" s="70" t="s">
+      <c r="E36" s="69" t="s">
         <v>23</v>
       </c>
-      <c r="I36" s="71"/>
-      <c r="J36" s="71"/>
+      <c r="I36" s="70"/>
+      <c r="J36" s="70"/>
     </row>
     <row r="37" spans="1:10" s="16" customFormat="1" ht="10.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A37" s="72" t="s">
+      <c r="A37" s="71" t="s">
         <v>6</v>
       </c>
-      <c r="B37" s="73"/>
-      <c r="C37" s="74" t="s">
+      <c r="B37" s="72"/>
+      <c r="C37" s="73" t="s">
         <v>24</v>
       </c>
-      <c r="D37" s="75"/>
-      <c r="E37" s="72" t="s">
+      <c r="D37" s="74"/>
+      <c r="E37" s="71" t="s">
         <v>6</v>
       </c>
-      <c r="F37" s="73"/>
-      <c r="G37" s="74" t="s">
+      <c r="F37" s="72"/>
+      <c r="G37" s="73" t="s">
         <v>25</v>
       </c>
-      <c r="I37" s="76"/>
-      <c r="J37" s="71"/>
+      <c r="I37" s="75"/>
+      <c r="J37" s="70"/>
     </row>
     <row r="38" spans="1:10" s="16" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="77"/>
-      <c r="B38" s="78"/>
-      <c r="C38" s="79"/>
-      <c r="D38" s="80"/>
-      <c r="E38" s="79"/>
-      <c r="F38" s="78"/>
-      <c r="G38" s="79"/>
-      <c r="H38" s="78"/>
-      <c r="I38" s="81"/>
-      <c r="J38" s="71"/>
+      <c r="A38" s="76"/>
+      <c r="B38" s="77"/>
+      <c r="C38" s="78"/>
+      <c r="D38" s="79"/>
+      <c r="E38" s="78"/>
+      <c r="F38" s="77"/>
+      <c r="G38" s="78"/>
+      <c r="H38" s="77"/>
+      <c r="I38" s="80"/>
+      <c r="J38" s="70"/>
     </row>
   </sheetData>
   <mergeCells count="4">

</xml_diff>